<commit_message>
docs: update product backlog with new scoring system PBIs
- Mark PBI-002, PBI-006, PBI-007, PBI-009 as Done
- Add PBI-032: Scoring Engine Redesign (Done, 8pts, Sprint 2)
- Add PBI-033: Engagement Score (To Do, 5pts, Sprint 3)
- Add PBI-034: Weekly Review Layer (To Do, 8pts, Sprint 3)
- Update Sprint 2 plan (26pts) and Sprint 3 plan (33pts)
- Update Epic Summary and totals (34 PBIs, 147pts)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BLNC_Product_Backlog.xlsx
+++ b/BLNC_Product_Backlog.xlsx
@@ -590,7 +590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" style="29" min="1" max="1"/>
@@ -726,7 +726,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H3" s="2" t="n"/>
@@ -901,7 +901,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H7" s="2" t="n"/>
@@ -945,7 +945,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H8" s="2" t="n"/>
@@ -1002,6 +1002,16 @@
 6. X-axis shows dates, Y-axis shows score 0-100</t>
         </is>
       </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>1. Line chart shows overall Balance Score over past 7 days, 30 days, and 90 days
+2. User can toggle between time ranges
+3. Individual domain scores can be overlaid or viewed separately
+4. Data sourced from dailySnapshots collection (saved on each check-in)
+5. Chart handles missing days gracefully (gap or interpolation)
+6. X-axis shows dates, Y-axis shows score 0-100</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="90" customHeight="1" s="29">
       <c r="A10" s="2" t="inlineStr">
@@ -1032,7 +1042,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H10" s="2" t="n"/>
@@ -1104,7 +1114,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>As a user, I want to receive 2-3 personalised weekly micro actions based on my weakest domains, so that I have clear, actionable guidance on what to focus on.</t>
+          <t>As a user, I want to receive 2-3 personalised weekly micro actions based on my weakest domains from the weekly review, so that I have clear, actionable guidance on what to focus on.</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1133,6 +1143,18 @@
 5. User can mark each action as completed or skipped
 6. Completing an action positively impacts the relevant domain score
 7. New actions are generated weekly, not repeated consecutively</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>1. Weekly review identifies the 1-2 weakest domains from domain scores
+2. App generates 2-3 micro actions targeting those domains
+3. Actions are specific and achievable (e.g. 'Take a 15-min walk today')
+4. Each action displays estimated time to complete
+5. Actions are tagged to their relevant domain
+6. User can mark each action as completed or skipped
+7. Completing an action contributes to today's action signal (30% of daily domain signal)
+8. New actions are generated weekly, not repeated consecutively</t>
         </is>
       </c>
     </row>
@@ -2011,6 +2033,144 @@
 8. Shared UI components created (Button, Card, Input, ScoreCircle, EmptyState)
 9. Theme config with colours, spacing, typography
 10. Feature folder structure scaffolded for all domains</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>PBI-032</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Balance Score &amp; Dashboard</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>As a developer, I want the scoring engine redesigned with geometric mean Balance Score, daily EMA updates, and anti-gaming protections, so that scores are responsive, stable, and fair.</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F33" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="n"/>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>1. Balance Score uses geometric mean of 5 domain scores (not arithmetic mean × factor)
+2. Zero-floor applied before geometric mean to prevent zero-collapse
+3. Daily check-in updates use EMA (α=0.12) for smooth, immediate score movement
+4. Daily movement capped at ±3 points per domain (anti-gaming)
+5. Check-in uses 1-5 scale mapped to 0-100 via ((value-1)/4)*100
+6. Assessment uses same formula: ((response-1)/4)*100
+7. Wellbeing and engagement are tracked separately
+8. Imbalance SD calculated for weekly insights
+9. Daily snapshots saved to Firestore for trend charts
+10. All 23 unit tests passing</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>PBI-033</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Balance Score &amp; Dashboard</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>As a user, I want a separate Engagement Score that tracks my app consistency, so that missing a day doesn't lower my wellbeing scores and I can see participation and wellbeing as distinct metrics.</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F34" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="n"/>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>1. Engagement Score displayed on dashboard alongside Balance Score
+2. Score formula: 40% check-in completion + 30% action completion + 20% streak + 10% feature use
+3. All components scaled to 0-100
+4. Engagement Score updates after each check-in or action
+5. Score does NOT affect domain or Balance Score
+6. Insights distinguish wellbeing from engagement (e.g. 'Your balance is steady but engagement dropped')</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>PBI-034</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Balance Score &amp; Dashboard</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>As a user, I want a weekly review summary that analyses my past 7 days, identifies trends, and triggers personalised mission generation, so that the app gives me intelligent insights beyond daily score movement.</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F35" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="n"/>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
+          <t>1. Weekly summary computed every Monday (or on-demand)
+2. Per-domain: average daily check-in score + action completion score
+3. Imbalance indicator (SD) identifies if user is balanced or uneven
+4. Strongest and weakest domains identified
+5. Trend direction shown (improving / declining / steady per domain)
+6. Weekly summary stored in Firestore for historical comparison
+7. Summary triggers weekly mission generation (PBI-011)
+8. Insights viewable on Progress tab</t>
         </is>
       </c>
     </row>
@@ -2115,15 +2275,15 @@
       </c>
       <c r="D3" s="11" t="inlineStr">
         <is>
-          <t>PBI-008, PBI-009, PBI-011</t>
+          <t>PBI-008, PBI-009, PBI-011, PBI-032</t>
         </is>
       </c>
       <c r="E3" s="10" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="F3" s="11" t="inlineStr">
         <is>
-          <t>Users can check in daily, receive weekly micro actions, and view score trends over time. Core engagement loop complete.</t>
+          <t>Users can check in daily with new 1-5 scale, scores update via EMA, view score trends over time, and receive weekly micro actions. Scoring engine redesigned with geometric mean and anti-gaming protections.</t>
         </is>
       </c>
     </row>
@@ -2145,15 +2305,15 @@
       <c r="D4" s="13" t="inlineStr">
         <is>
           <t>PBI-010, PBI-012, PBI-013,
-PBI-015, PBI-016, PBI-021</t>
+PBI-015, PBI-016, PBI-021, PBI-033, PBI-034</t>
         </is>
       </c>
       <c r="E4" s="12" t="n">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="F4" s="13" t="inlineStr">
         <is>
-          <t>Mood tracker, journal, to-do list, streaks, and check-in reminders working. Mental health and productivity domains have dedicated tracking.</t>
+          <t>Engagement Score, weekly review layer, mood tracker, journal, to-do list, streaks, and check-in reminders. Mental health and productivity domains have dedicated tracking. Weekly insights drive mission generation.</t>
         </is>
       </c>
     </row>
@@ -2343,23 +2503,23 @@
         </is>
       </c>
       <c r="B3" s="20" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C3" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D3" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E3" s="20" t="n">
         <v>0</v>
       </c>
       <c r="F3" s="20" t="n">
-        <v>18</v>
+        <v>39</v>
       </c>
       <c r="G3" s="20" t="inlineStr">
         <is>
-          <t>1, 2</t>
+          <t>1, 2, 3</t>
         </is>
       </c>
     </row>
@@ -2667,10 +2827,10 @@
         </is>
       </c>
       <c r="B15" s="21" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C15" s="21" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D15" s="21">
         <f>SUM(D2:D13)</f>
@@ -2681,7 +2841,7 @@
         <v/>
       </c>
       <c r="F15" s="21" t="n">
-        <v>126</v>
+        <v>147</v>
       </c>
       <c r="G15" s="21" t="n"/>
     </row>

</xml_diff>